<commit_message>
update: modify inventory/sales import template
</commit_message>
<xml_diff>
--- a/static/templates/SmartVenta_plantilla_importacion_inventario_o_ventas.xlsx
+++ b/static/templates/SmartVenta_plantilla_importacion_inventario_o_ventas.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
   <si>
     <t xml:space="preserve">Código</t>
   </si>
@@ -38,10 +38,22 @@
     <t xml:space="preserve">Opcional</t>
   </si>
   <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
     <t xml:space="preserve">Agua 1l</t>
   </si>
   <si>
+    <t xml:space="preserve">2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Agua 2l</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refresco</t>
   </si>
 </sst>
 </file>
@@ -186,7 +198,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9.2"/>
@@ -265,7 +277,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultColWidth="8.37890625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="11.22"/>
@@ -313,28 +325,39 @@
       <c r="I2" s="5"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
-        <v>1</v>
+      <c r="A3" s="0" t="s">
+        <v>5</v>
       </c>
       <c r="B3" s="0" t="n">
         <v>1</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
-        <v>1</v>
+      <c r="A4" s="0" t="s">
+        <v>7</v>
       </c>
       <c r="B4" s="0" t="n">
         <v>2</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I4" s="3"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>